<commit_message>
Refresh sector data 2026-10-12
</commit_message>
<xml_diff>
--- a/data/sectoraldata.xlsx
+++ b/data/sectoraldata.xlsx
@@ -5863,7 +5863,7 @@
         <v>0.1069</v>
       </c>
       <c r="L63" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="M63" t="n">
         <v>0.0137</v>
@@ -23267,7 +23267,7 @@
         <v>0.0193</v>
       </c>
       <c r="N421" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="O421" t="n">
         <v>-0.0028</v>
@@ -29809,7 +29809,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1897; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1897; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -30377,7 +30377,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1926; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1926; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -30945,7 +30945,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1901; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1901; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -31513,7 +31513,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1904; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1904; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -32081,7 +32081,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1898; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1898; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -32649,7 +32649,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1906; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1906; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -33217,7 +33217,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 910338; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 910338; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -33785,7 +33785,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 910396; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 910396; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -34161,7 +34161,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1896; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1896; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G17" s="4" t="n"/>
@@ -34430,7 +34430,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 910398; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 910398; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G12" s="4" t="n"/>
@@ -34998,7 +34998,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1887; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1887; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -35566,7 +35566,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1894; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1894; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -35942,7 +35942,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1895; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1895; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G17" s="4" t="n"/>
@@ -36510,7 +36510,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 910393; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 910393; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -37078,7 +37078,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 910414; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 910414; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -37640,7 +37640,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1907; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1907; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -38208,7 +38208,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1908; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1908; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -38776,7 +38776,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 910411; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 910411; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -39344,7 +39344,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1910; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1910; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -39404,7 +39404,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -39426,7 +39426,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -39448,7 +39448,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -39470,7 +39470,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -39492,7 +39492,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -39514,7 +39514,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -39536,7 +39536,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -39558,7 +39558,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -39580,7 +39580,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -39602,7 +39602,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -39624,7 +39624,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -39646,7 +39646,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -39668,7 +39668,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -39690,7 +39690,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -39712,7 +39712,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -39734,7 +39734,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -39756,7 +39756,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -39778,7 +39778,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -39800,7 +39800,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -39822,7 +39822,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -39844,7 +39844,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -39866,7 +39866,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -39888,7 +39888,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -39910,7 +39910,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -39932,7 +39932,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -39954,7 +39954,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -40012,7 +40012,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -40034,7 +40034,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -40056,7 +40056,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -40078,7 +40078,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -40100,7 +40100,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -40122,7 +40122,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -40144,7 +40144,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -40166,7 +40166,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -40188,7 +40188,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -40210,7 +40210,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -40232,7 +40232,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -40254,7 +40254,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -40276,7 +40276,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -40298,7 +40298,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -40320,7 +40320,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -40342,7 +40342,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -40364,7 +40364,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -40386,7 +40386,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -40408,7 +40408,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -40430,7 +40430,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -40452,7 +40452,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -40474,7 +40474,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -40496,7 +40496,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -40518,7 +40518,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -40540,7 +40540,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -40562,7 +40562,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>fresh</t>
+          <t>cached</t>
         </is>
       </c>
     </row>
@@ -41128,7 +41128,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1888; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1888; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -41696,7 +41696,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1902; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1902; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -42264,7 +42264,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1911; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1911; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -42832,7 +42832,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1909; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1909; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -43400,7 +43400,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1899; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1899; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -43968,7 +43968,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 910417; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 910417; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -44536,7 +44536,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1905; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1905; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>

</xml_diff>